<commit_message>
Remove Middletown from payroll GL export
- Removed the Middeltown column (AC) from data/allocation.xlsx so it no
  longer appears as a property row in any payroll or GL export
- Removed the Middeltown entry from the property name mapping table in
  the same workbook
- Updated Harry Feldman's allocation note to reflect the split is now
  between Interstate and Eastwick only (Middletown removed)

The export totals dynamically sum the remaining property rows, so the
grand total will balance correctly without Middletown.

https://claude.ai/code/session_01T6k9QDiM96YPHaboHxNHuD
</commit_message>
<xml_diff>
--- a/data/allocation.xlsx
+++ b/data/allocation.xlsx
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AN95"/>
+  <dimension ref="A1:AM94"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -488,10 +488,10 @@
         <v>0800</v>
       </c>
       <c r="AC1" t="str">
-        <v>Middeltown</v>
+        <v>Eastwick</v>
       </c>
       <c r="AD1" t="str">
-        <v>Eastwick</v>
+        <v/>
       </c>
       <c r="AE1" t="str">
         <v/>
@@ -503,24 +503,21 @@
         <v/>
       </c>
       <c r="AH1" t="str">
-        <v/>
+        <v>JV III</v>
       </c>
       <c r="AI1" t="str">
-        <v>JV III</v>
+        <v xml:space="preserve"> NI LLC</v>
       </c>
       <c r="AJ1" t="str">
-        <v xml:space="preserve"> NI LLC</v>
+        <v>SC</v>
       </c>
       <c r="AK1" t="str">
-        <v>SC</v>
+        <v/>
       </c>
       <c r="AL1" t="str">
         <v/>
       </c>
       <c r="AM1" t="str">
-        <v/>
-      </c>
-      <c r="AN1" t="str">
         <v/>
       </c>
     </row>
@@ -613,7 +610,7 @@
         <v>0</v>
       </c>
       <c r="AD2" t="str">
-        <v>0</v>
+        <v/>
       </c>
       <c r="AE2" t="str">
         <v/>
@@ -625,24 +622,21 @@
         <v/>
       </c>
       <c r="AH2" t="str">
-        <v/>
+        <v>0.1141</v>
       </c>
       <c r="AI2" t="str">
-        <v>0.1141</v>
+        <v>0.2359</v>
       </c>
       <c r="AJ2" t="str">
-        <v>0.2359</v>
+        <v>0.35</v>
       </c>
       <c r="AK2" t="str">
-        <v>0.35</v>
+        <v/>
       </c>
       <c r="AL2" t="str">
         <v/>
       </c>
       <c r="AM2" t="str">
-        <v/>
-      </c>
-      <c r="AN2" t="str">
         <v/>
       </c>
     </row>
@@ -764,9 +758,6 @@
       <c r="AM3" t="str">
         <v/>
       </c>
-      <c r="AN3" t="str">
-        <v/>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -857,7 +848,7 @@
         <v>0</v>
       </c>
       <c r="AD4" t="str">
-        <v>0</v>
+        <v/>
       </c>
       <c r="AE4" t="str">
         <v/>
@@ -869,7 +860,7 @@
         <v/>
       </c>
       <c r="AH4" t="str">
-        <v/>
+        <v>0</v>
       </c>
       <c r="AI4" t="str">
         <v>0</v>
@@ -878,15 +869,12 @@
         <v>0</v>
       </c>
       <c r="AK4" t="str">
-        <v>0</v>
+        <v/>
       </c>
       <c r="AL4" t="str">
         <v/>
       </c>
       <c r="AM4" t="str">
-        <v/>
-      </c>
-      <c r="AN4" t="str">
         <v/>
       </c>
     </row>
@@ -979,7 +967,7 @@
         <v>0</v>
       </c>
       <c r="AD5" t="str">
-        <v>0</v>
+        <v/>
       </c>
       <c r="AE5" t="str">
         <v/>
@@ -991,7 +979,7 @@
         <v/>
       </c>
       <c r="AH5" t="str">
-        <v/>
+        <v>0</v>
       </c>
       <c r="AI5" t="str">
         <v>0</v>
@@ -1000,15 +988,12 @@
         <v>0</v>
       </c>
       <c r="AK5" t="str">
-        <v>0</v>
+        <v/>
       </c>
       <c r="AL5" t="str">
         <v/>
       </c>
       <c r="AM5" t="str">
-        <v/>
-      </c>
-      <c r="AN5" t="str">
         <v/>
       </c>
     </row>
@@ -1101,7 +1086,7 @@
         <v>0</v>
       </c>
       <c r="AD6" t="str">
-        <v>0</v>
+        <v/>
       </c>
       <c r="AE6" t="str">
         <v/>
@@ -1113,7 +1098,7 @@
         <v/>
       </c>
       <c r="AH6" t="str">
-        <v/>
+        <v>0</v>
       </c>
       <c r="AI6" t="str">
         <v>0</v>
@@ -1122,15 +1107,12 @@
         <v>0</v>
       </c>
       <c r="AK6" t="str">
-        <v>0</v>
+        <v/>
       </c>
       <c r="AL6" t="str">
         <v/>
       </c>
       <c r="AM6" t="str">
-        <v/>
-      </c>
-      <c r="AN6" t="str">
         <v/>
       </c>
     </row>
@@ -1223,7 +1205,7 @@
         <v>0</v>
       </c>
       <c r="AD7" t="str">
-        <v>0</v>
+        <v/>
       </c>
       <c r="AE7" t="str">
         <v/>
@@ -1235,7 +1217,7 @@
         <v/>
       </c>
       <c r="AH7" t="str">
-        <v/>
+        <v>0</v>
       </c>
       <c r="AI7" t="str">
         <v>0</v>
@@ -1244,15 +1226,12 @@
         <v>0</v>
       </c>
       <c r="AK7" t="str">
-        <v>0</v>
+        <v/>
       </c>
       <c r="AL7" t="str">
         <v/>
       </c>
       <c r="AM7" t="str">
-        <v/>
-      </c>
-      <c r="AN7" t="str">
         <v/>
       </c>
     </row>
@@ -1345,7 +1324,7 @@
         <v>0</v>
       </c>
       <c r="AD8" t="str">
-        <v>0</v>
+        <v/>
       </c>
       <c r="AE8" t="str">
         <v/>
@@ -1357,7 +1336,7 @@
         <v/>
       </c>
       <c r="AH8" t="str">
-        <v/>
+        <v>0</v>
       </c>
       <c r="AI8" t="str">
         <v>0</v>
@@ -1366,15 +1345,12 @@
         <v>0</v>
       </c>
       <c r="AK8" t="str">
-        <v>0</v>
+        <v/>
       </c>
       <c r="AL8" t="str">
         <v/>
       </c>
       <c r="AM8" t="str">
-        <v/>
-      </c>
-      <c r="AN8" t="str">
         <v/>
       </c>
     </row>
@@ -1467,7 +1443,7 @@
         <v>0.051367618</v>
       </c>
       <c r="AD9" t="str">
-        <v>0.051367618</v>
+        <v/>
       </c>
       <c r="AE9" t="str">
         <v/>
@@ -1479,24 +1455,21 @@
         <v/>
       </c>
       <c r="AH9" t="str">
-        <v/>
+        <v>0</v>
       </c>
       <c r="AI9" t="str">
         <v>0</v>
       </c>
       <c r="AJ9" t="str">
-        <v>0</v>
+        <v>0.845897146</v>
       </c>
       <c r="AK9" t="str">
-        <v>0.845897146</v>
+        <v/>
       </c>
       <c r="AL9" t="str">
         <v/>
       </c>
       <c r="AM9" t="str">
-        <v/>
-      </c>
-      <c r="AN9" t="str">
         <v/>
       </c>
     </row>
@@ -1589,7 +1562,7 @@
         <v>0</v>
       </c>
       <c r="AD10" t="str">
-        <v>0</v>
+        <v/>
       </c>
       <c r="AE10" t="str">
         <v/>
@@ -1601,24 +1574,21 @@
         <v/>
       </c>
       <c r="AH10" t="str">
-        <v/>
+        <v>0.163</v>
       </c>
       <c r="AI10" t="str">
-        <v>0.163</v>
+        <v>0.337</v>
       </c>
       <c r="AJ10" t="str">
-        <v>0.337</v>
+        <v>0.5</v>
       </c>
       <c r="AK10" t="str">
-        <v>0.5</v>
+        <v/>
       </c>
       <c r="AL10" t="str">
         <v/>
       </c>
       <c r="AM10" t="str">
-        <v/>
-      </c>
-      <c r="AN10" t="str">
         <v/>
       </c>
     </row>
@@ -1711,7 +1681,7 @@
         <v>0</v>
       </c>
       <c r="AD11" t="str">
-        <v>0</v>
+        <v/>
       </c>
       <c r="AE11" t="str">
         <v/>
@@ -1723,24 +1693,21 @@
         <v/>
       </c>
       <c r="AH11" t="str">
-        <v/>
+        <v>0.163</v>
       </c>
       <c r="AI11" t="str">
-        <v>0.163</v>
+        <v>0.337</v>
       </c>
       <c r="AJ11" t="str">
-        <v>0.337</v>
+        <v>0.5</v>
       </c>
       <c r="AK11" t="str">
-        <v>0.5</v>
+        <v/>
       </c>
       <c r="AL11" t="str">
         <v/>
       </c>
       <c r="AM11" t="str">
-        <v/>
-      </c>
-      <c r="AN11" t="str">
         <v/>
       </c>
     </row>
@@ -1833,7 +1800,7 @@
         <v>0</v>
       </c>
       <c r="AD12" t="str">
-        <v>0</v>
+        <v/>
       </c>
       <c r="AE12" t="str">
         <v/>
@@ -1845,24 +1812,21 @@
         <v/>
       </c>
       <c r="AH12" t="str">
-        <v/>
+        <v>0.163</v>
       </c>
       <c r="AI12" t="str">
-        <v>0.163</v>
+        <v>0.337</v>
       </c>
       <c r="AJ12" t="str">
-        <v>0.337</v>
+        <v>0.5</v>
       </c>
       <c r="AK12" t="str">
-        <v>0.5</v>
+        <v/>
       </c>
       <c r="AL12" t="str">
         <v/>
       </c>
       <c r="AM12" t="str">
-        <v/>
-      </c>
-      <c r="AN12" t="str">
         <v/>
       </c>
     </row>
@@ -1955,7 +1919,7 @@
         <v>0</v>
       </c>
       <c r="AD13" t="str">
-        <v>0</v>
+        <v/>
       </c>
       <c r="AE13" t="str">
         <v/>
@@ -1967,24 +1931,21 @@
         <v/>
       </c>
       <c r="AH13" t="str">
-        <v/>
+        <v>0.2934</v>
       </c>
       <c r="AI13" t="str">
-        <v>0.2934</v>
+        <v>0.6066</v>
       </c>
       <c r="AJ13" t="str">
-        <v>0.6066</v>
+        <v>0</v>
       </c>
       <c r="AK13" t="str">
-        <v>0</v>
+        <v/>
       </c>
       <c r="AL13" t="str">
         <v/>
       </c>
       <c r="AM13" t="str">
-        <v/>
-      </c>
-      <c r="AN13" t="str">
         <v/>
       </c>
     </row>
@@ -2077,7 +2038,7 @@
         <v>0</v>
       </c>
       <c r="AD14" t="str">
-        <v>0</v>
+        <v/>
       </c>
       <c r="AE14" t="str">
         <v/>
@@ -2089,24 +2050,21 @@
         <v/>
       </c>
       <c r="AH14" t="str">
-        <v/>
+        <v>0.2119</v>
       </c>
       <c r="AI14" t="str">
-        <v>0.2119</v>
+        <v>0.4381</v>
       </c>
       <c r="AJ14" t="str">
-        <v>0.4381</v>
+        <v>0.35</v>
       </c>
       <c r="AK14" t="str">
-        <v>0.35</v>
+        <v/>
       </c>
       <c r="AL14" t="str">
         <v/>
       </c>
       <c r="AM14" t="str">
-        <v/>
-      </c>
-      <c r="AN14" t="str">
         <v/>
       </c>
     </row>
@@ -2199,7 +2157,7 @@
         <v>0</v>
       </c>
       <c r="AD15" t="str">
-        <v>0</v>
+        <v/>
       </c>
       <c r="AE15" t="str">
         <v/>
@@ -2211,24 +2169,21 @@
         <v/>
       </c>
       <c r="AH15" t="str">
-        <v/>
+        <v>0.163</v>
       </c>
       <c r="AI15" t="str">
-        <v>0.163</v>
+        <v>0.337</v>
       </c>
       <c r="AJ15" t="str">
-        <v>0.337</v>
+        <v>0.5</v>
       </c>
       <c r="AK15" t="str">
-        <v>0.5</v>
+        <v/>
       </c>
       <c r="AL15" t="str">
         <v/>
       </c>
       <c r="AM15" t="str">
-        <v/>
-      </c>
-      <c r="AN15" t="str">
         <v/>
       </c>
     </row>
@@ -2350,9 +2305,6 @@
       <c r="AM16" t="str">
         <v/>
       </c>
-      <c r="AN16" t="str">
-        <v/>
-      </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
@@ -2472,9 +2424,6 @@
       <c r="AM17" t="str">
         <v/>
       </c>
-      <c r="AN17" t="str">
-        <v/>
-      </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
@@ -2594,9 +2543,6 @@
       <c r="AM18" t="str">
         <v/>
       </c>
-      <c r="AN18" t="str">
-        <v/>
-      </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
@@ -2716,9 +2662,6 @@
       <c r="AM19" t="str">
         <v/>
       </c>
-      <c r="AN19" t="str">
-        <v/>
-      </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
@@ -2838,9 +2781,6 @@
       <c r="AM20" t="str">
         <v/>
       </c>
-      <c r="AN20" t="str">
-        <v/>
-      </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
@@ -2960,9 +2900,6 @@
       <c r="AM21" t="str">
         <v/>
       </c>
-      <c r="AN21" t="str">
-        <v/>
-      </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
@@ -3082,9 +3019,6 @@
       <c r="AM22" t="str">
         <v/>
       </c>
-      <c r="AN22" t="str">
-        <v/>
-      </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
@@ -3204,9 +3138,6 @@
       <c r="AM23" t="str">
         <v/>
       </c>
-      <c r="AN23" t="str">
-        <v/>
-      </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
@@ -3326,9 +3257,6 @@
       <c r="AM24" t="str">
         <v/>
       </c>
-      <c r="AN24" t="str">
-        <v/>
-      </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
@@ -3448,9 +3376,6 @@
       <c r="AM25" t="str">
         <v/>
       </c>
-      <c r="AN25" t="str">
-        <v/>
-      </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
@@ -3570,9 +3495,6 @@
       <c r="AM26" t="str">
         <v/>
       </c>
-      <c r="AN26" t="str">
-        <v/>
-      </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
@@ -3692,9 +3614,6 @@
       <c r="AM27" t="str">
         <v/>
       </c>
-      <c r="AN27" t="str">
-        <v/>
-      </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
@@ -3814,9 +3733,6 @@
       <c r="AM28" t="str">
         <v/>
       </c>
-      <c r="AN28" t="str">
-        <v/>
-      </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
@@ -3936,9 +3852,6 @@
       <c r="AM29" t="str">
         <v/>
       </c>
-      <c r="AN29" t="str">
-        <v/>
-      </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
@@ -4058,9 +3971,6 @@
       <c r="AM30" t="str">
         <v/>
       </c>
-      <c r="AN30" t="str">
-        <v/>
-      </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
@@ -4180,9 +4090,6 @@
       <c r="AM31" t="str">
         <v/>
       </c>
-      <c r="AN31" t="str">
-        <v/>
-      </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
@@ -4302,9 +4209,6 @@
       <c r="AM32" t="str">
         <v/>
       </c>
-      <c r="AN32" t="str">
-        <v/>
-      </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
@@ -4424,9 +4328,6 @@
       <c r="AM33" t="str">
         <v/>
       </c>
-      <c r="AN33" t="str">
-        <v/>
-      </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
@@ -4546,9 +4447,6 @@
       <c r="AM34" t="str">
         <v/>
       </c>
-      <c r="AN34" t="str">
-        <v/>
-      </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
@@ -4668,9 +4566,6 @@
       <c r="AM35" t="str">
         <v/>
       </c>
-      <c r="AN35" t="str">
-        <v/>
-      </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
@@ -4790,9 +4685,6 @@
       <c r="AM36" t="str">
         <v/>
       </c>
-      <c r="AN36" t="str">
-        <v/>
-      </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
@@ -4912,9 +4804,6 @@
       <c r="AM37" t="str">
         <v/>
       </c>
-      <c r="AN37" t="str">
-        <v/>
-      </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
@@ -5034,9 +4923,6 @@
       <c r="AM38" t="str">
         <v/>
       </c>
-      <c r="AN38" t="str">
-        <v/>
-      </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
@@ -5156,9 +5042,6 @@
       <c r="AM39" t="str">
         <v/>
       </c>
-      <c r="AN39" t="str">
-        <v/>
-      </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
@@ -5278,9 +5161,6 @@
       <c r="AM40" t="str">
         <v/>
       </c>
-      <c r="AN40" t="str">
-        <v/>
-      </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
@@ -5400,9 +5280,6 @@
       <c r="AM41" t="str">
         <v/>
       </c>
-      <c r="AN41" t="str">
-        <v/>
-      </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
@@ -5522,9 +5399,6 @@
       <c r="AM42" t="str">
         <v/>
       </c>
-      <c r="AN42" t="str">
-        <v/>
-      </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
@@ -5644,9 +5518,6 @@
       <c r="AM43" t="str">
         <v/>
       </c>
-      <c r="AN43" t="str">
-        <v/>
-      </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
@@ -5766,9 +5637,6 @@
       <c r="AM44" t="str">
         <v/>
       </c>
-      <c r="AN44" t="str">
-        <v/>
-      </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
@@ -5888,9 +5756,6 @@
       <c r="AM45" t="str">
         <v/>
       </c>
-      <c r="AN45" t="str">
-        <v/>
-      </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
@@ -6010,9 +5875,6 @@
       <c r="AM46" t="str">
         <v/>
       </c>
-      <c r="AN46" t="str">
-        <v/>
-      </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
@@ -6132,9 +5994,6 @@
       <c r="AM47" t="str">
         <v/>
       </c>
-      <c r="AN47" t="str">
-        <v/>
-      </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
@@ -6254,9 +6113,6 @@
       <c r="AM48" t="str">
         <v/>
       </c>
-      <c r="AN48" t="str">
-        <v/>
-      </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
@@ -6376,9 +6232,6 @@
       <c r="AM49" t="str">
         <v/>
       </c>
-      <c r="AN49" t="str">
-        <v/>
-      </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
@@ -6498,9 +6351,6 @@
       <c r="AM50" t="str">
         <v/>
       </c>
-      <c r="AN50" t="str">
-        <v/>
-      </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
@@ -6620,9 +6470,6 @@
       <c r="AM51" t="str">
         <v/>
       </c>
-      <c r="AN51" t="str">
-        <v/>
-      </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
@@ -6742,9 +6589,6 @@
       <c r="AM52" t="str">
         <v/>
       </c>
-      <c r="AN52" t="str">
-        <v/>
-      </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
@@ -6864,9 +6708,6 @@
       <c r="AM53" t="str">
         <v/>
       </c>
-      <c r="AN53" t="str">
-        <v/>
-      </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
@@ -6986,9 +6827,6 @@
       <c r="AM54" t="str">
         <v/>
       </c>
-      <c r="AN54" t="str">
-        <v/>
-      </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
@@ -7108,9 +6946,6 @@
       <c r="AM55" t="str">
         <v/>
       </c>
-      <c r="AN55" t="str">
-        <v/>
-      </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
@@ -7230,9 +7065,6 @@
       <c r="AM56" t="str">
         <v/>
       </c>
-      <c r="AN56" t="str">
-        <v/>
-      </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
@@ -7352,9 +7184,6 @@
       <c r="AM57" t="str">
         <v/>
       </c>
-      <c r="AN57" t="str">
-        <v/>
-      </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
@@ -7474,9 +7303,6 @@
       <c r="AM58" t="str">
         <v/>
       </c>
-      <c r="AN58" t="str">
-        <v/>
-      </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
@@ -7596,9 +7422,6 @@
       <c r="AM59" t="str">
         <v/>
       </c>
-      <c r="AN59" t="str">
-        <v/>
-      </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
@@ -7718,9 +7541,6 @@
       <c r="AM60" t="str">
         <v/>
       </c>
-      <c r="AN60" t="str">
-        <v/>
-      </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
@@ -7840,9 +7660,6 @@
       <c r="AM61" t="str">
         <v/>
       </c>
-      <c r="AN61" t="str">
-        <v/>
-      </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
@@ -7962,9 +7779,6 @@
       <c r="AM62" t="str">
         <v/>
       </c>
-      <c r="AN62" t="str">
-        <v/>
-      </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
@@ -8084,9 +7898,6 @@
       <c r="AM63" t="str">
         <v/>
       </c>
-      <c r="AN63" t="str">
-        <v/>
-      </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
@@ -8206,9 +8017,6 @@
       <c r="AM64" t="str">
         <v/>
       </c>
-      <c r="AN64" t="str">
-        <v/>
-      </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
@@ -8328,9 +8136,6 @@
       <c r="AM65" t="str">
         <v/>
       </c>
-      <c r="AN65" t="str">
-        <v/>
-      </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
@@ -8450,9 +8255,6 @@
       <c r="AM66" t="str">
         <v/>
       </c>
-      <c r="AN66" t="str">
-        <v/>
-      </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
@@ -8572,9 +8374,6 @@
       <c r="AM67" t="str">
         <v/>
       </c>
-      <c r="AN67" t="str">
-        <v/>
-      </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
@@ -8694,9 +8493,6 @@
       <c r="AM68" t="str">
         <v/>
       </c>
-      <c r="AN68" t="str">
-        <v/>
-      </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
@@ -8816,9 +8612,6 @@
       <c r="AM69" t="str">
         <v/>
       </c>
-      <c r="AN69" t="str">
-        <v/>
-      </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
@@ -8938,9 +8731,6 @@
       <c r="AM70" t="str">
         <v/>
       </c>
-      <c r="AN70" t="str">
-        <v/>
-      </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
@@ -9060,9 +8850,6 @@
       <c r="AM71" t="str">
         <v/>
       </c>
-      <c r="AN71" t="str">
-        <v/>
-      </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
@@ -9182,9 +8969,6 @@
       <c r="AM72" t="str">
         <v/>
       </c>
-      <c r="AN72" t="str">
-        <v/>
-      </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
@@ -9304,9 +9088,6 @@
       <c r="AM73" t="str">
         <v/>
       </c>
-      <c r="AN73" t="str">
-        <v/>
-      </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
@@ -9426,9 +9207,6 @@
       <c r="AM74" t="str">
         <v/>
       </c>
-      <c r="AN74" t="str">
-        <v/>
-      </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
@@ -9548,9 +9326,6 @@
       <c r="AM75" t="str">
         <v/>
       </c>
-      <c r="AN75" t="str">
-        <v/>
-      </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
@@ -9670,9 +9445,6 @@
       <c r="AM76" t="str">
         <v/>
       </c>
-      <c r="AN76" t="str">
-        <v/>
-      </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
@@ -9792,9 +9564,6 @@
       <c r="AM77" t="str">
         <v/>
       </c>
-      <c r="AN77" t="str">
-        <v/>
-      </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
@@ -9914,9 +9683,6 @@
       <c r="AM78" t="str">
         <v/>
       </c>
-      <c r="AN78" t="str">
-        <v/>
-      </c>
     </row>
     <row r="79">
       <c r="A79" t="str">
@@ -10036,9 +9802,6 @@
       <c r="AM79" t="str">
         <v/>
       </c>
-      <c r="AN79" t="str">
-        <v/>
-      </c>
     </row>
     <row r="80">
       <c r="A80" t="str">
@@ -10158,9 +9921,6 @@
       <c r="AM80" t="str">
         <v/>
       </c>
-      <c r="AN80" t="str">
-        <v/>
-      </c>
     </row>
     <row r="81">
       <c r="A81" t="str">
@@ -10280,9 +10040,6 @@
       <c r="AM81" t="str">
         <v/>
       </c>
-      <c r="AN81" t="str">
-        <v/>
-      </c>
     </row>
     <row r="82">
       <c r="A82" t="str">
@@ -10402,9 +10159,6 @@
       <c r="AM82" t="str">
         <v/>
       </c>
-      <c r="AN82" t="str">
-        <v/>
-      </c>
     </row>
     <row r="83">
       <c r="A83" t="str">
@@ -10524,9 +10278,6 @@
       <c r="AM83" t="str">
         <v/>
       </c>
-      <c r="AN83" t="str">
-        <v/>
-      </c>
     </row>
     <row r="84">
       <c r="A84" t="str">
@@ -10646,9 +10397,6 @@
       <c r="AM84" t="str">
         <v/>
       </c>
-      <c r="AN84" t="str">
-        <v/>
-      </c>
     </row>
     <row r="85">
       <c r="A85" t="str">
@@ -10768,9 +10516,6 @@
       <c r="AM85" t="str">
         <v/>
       </c>
-      <c r="AN85" t="str">
-        <v/>
-      </c>
     </row>
     <row r="86">
       <c r="A86" t="str">
@@ -10890,9 +10635,6 @@
       <c r="AM86" t="str">
         <v/>
       </c>
-      <c r="AN86" t="str">
-        <v/>
-      </c>
     </row>
     <row r="87">
       <c r="A87" t="str">
@@ -11012,9 +10754,6 @@
       <c r="AM87" t="str">
         <v/>
       </c>
-      <c r="AN87" t="str">
-        <v/>
-      </c>
     </row>
     <row r="88">
       <c r="A88" t="str">
@@ -11134,9 +10873,6 @@
       <c r="AM88" t="str">
         <v/>
       </c>
-      <c r="AN88" t="str">
-        <v/>
-      </c>
     </row>
     <row r="89">
       <c r="A89" t="str">
@@ -11256,9 +10992,6 @@
       <c r="AM89" t="str">
         <v/>
       </c>
-      <c r="AN89" t="str">
-        <v/>
-      </c>
     </row>
     <row r="90">
       <c r="A90" t="str">
@@ -11378,9 +11111,6 @@
       <c r="AM90" t="str">
         <v/>
       </c>
-      <c r="AN90" t="str">
-        <v/>
-      </c>
     </row>
     <row r="91">
       <c r="A91" t="str">
@@ -11500,9 +11230,6 @@
       <c r="AM91" t="str">
         <v/>
       </c>
-      <c r="AN91" t="str">
-        <v/>
-      </c>
     </row>
     <row r="92">
       <c r="A92" t="str">
@@ -11622,19 +11349,16 @@
       <c r="AM92" t="str">
         <v/>
       </c>
-      <c r="AN92" t="str">
-        <v/>
-      </c>
     </row>
     <row r="93">
       <c r="A93" t="str">
         <v/>
       </c>
       <c r="B93" t="str">
-        <v>Middeltown</v>
+        <v>Eastwick</v>
       </c>
       <c r="C93" t="str">
-        <v>Middletown</v>
+        <v>Eastwick JV</v>
       </c>
       <c r="D93" t="str">
         <v>0</v>
@@ -11742,9 +11466,6 @@
         <v/>
       </c>
       <c r="AM93" t="str">
-        <v/>
-      </c>
-      <c r="AN93" t="str">
         <v/>
       </c>
     </row>
@@ -11753,16 +11474,16 @@
         <v/>
       </c>
       <c r="B94" t="str">
-        <v>Eastwick</v>
+        <v/>
       </c>
       <c r="C94" t="str">
-        <v>Eastwick JV</v>
+        <v/>
       </c>
       <c r="D94" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E94" t="str">
-        <v>0</v>
+        <v>8568.95</v>
       </c>
       <c r="F94" t="str">
         <v/>
@@ -11864,137 +11585,12 @@
         <v/>
       </c>
       <c r="AM94" t="str">
-        <v/>
-      </c>
-      <c r="AN94" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95" t="str">
-        <v/>
-      </c>
-      <c r="B95" t="str">
-        <v/>
-      </c>
-      <c r="C95" t="str">
-        <v/>
-      </c>
-      <c r="D95" t="str">
-        <v>1</v>
-      </c>
-      <c r="E95" t="str">
-        <v>8568.95</v>
-      </c>
-      <c r="F95" t="str">
-        <v/>
-      </c>
-      <c r="G95" t="str">
-        <v/>
-      </c>
-      <c r="H95" t="str">
-        <v/>
-      </c>
-      <c r="I95" t="str">
-        <v/>
-      </c>
-      <c r="J95" t="str">
-        <v/>
-      </c>
-      <c r="K95" t="str">
-        <v/>
-      </c>
-      <c r="L95" t="str">
-        <v/>
-      </c>
-      <c r="M95" t="str">
-        <v/>
-      </c>
-      <c r="N95" t="str">
-        <v/>
-      </c>
-      <c r="O95" t="str">
-        <v/>
-      </c>
-      <c r="P95" t="str">
-        <v/>
-      </c>
-      <c r="Q95" t="str">
-        <v/>
-      </c>
-      <c r="R95" t="str">
-        <v/>
-      </c>
-      <c r="S95" t="str">
-        <v/>
-      </c>
-      <c r="T95" t="str">
-        <v/>
-      </c>
-      <c r="U95" t="str">
-        <v/>
-      </c>
-      <c r="V95" t="str">
-        <v/>
-      </c>
-      <c r="W95" t="str">
-        <v/>
-      </c>
-      <c r="X95" t="str">
-        <v/>
-      </c>
-      <c r="Y95" t="str">
-        <v/>
-      </c>
-      <c r="Z95" t="str">
-        <v/>
-      </c>
-      <c r="AA95" t="str">
-        <v/>
-      </c>
-      <c r="AB95" t="str">
-        <v/>
-      </c>
-      <c r="AC95" t="str">
-        <v/>
-      </c>
-      <c r="AD95" t="str">
-        <v/>
-      </c>
-      <c r="AE95" t="str">
-        <v/>
-      </c>
-      <c r="AF95" t="str">
-        <v/>
-      </c>
-      <c r="AG95" t="str">
-        <v/>
-      </c>
-      <c r="AH95" t="str">
-        <v/>
-      </c>
-      <c r="AI95" t="str">
-        <v/>
-      </c>
-      <c r="AJ95" t="str">
-        <v/>
-      </c>
-      <c r="AK95" t="str">
-        <v/>
-      </c>
-      <c r="AL95" t="str">
-        <v/>
-      </c>
-      <c r="AM95" t="str">
-        <v/>
-      </c>
-      <c r="AN95" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AN95"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AM94"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Payroll Invoicer: let Harry run it; add Stacie McShane allocation
- Drop the extra admin-auth gate on /api/parse-payroll, /api/allocation,
  /api/generate-all, /api/generate-pdf. These are pure-compute endpoints
  (no persistence) and the page is already restricted by per-user nav
  keys; the gate was rejecting Harry with "Unauthorized" when he tried
  to import a payroll file. /history and /api/periods still admin-gated.
- Add Stacie McShane (employee #34) to data/allocation.xlsx with the
  same property/fund allocation percentages as Marie Morsa-Jaster.

https://claude.ai/code/session_015kpdDzSngXqVmNwhqp8cqW
</commit_message>
<xml_diff>
--- a/data/allocation.xlsx
+++ b/data/allocation.xlsx
@@ -124,10 +124,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
+        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
+        <a:font script="Hans" typeface="å®ä½"/>
+        <a:font script="Hant" typeface="æ°ç´°æé«"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -159,10 +159,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
+        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
+        <a:font script="Hans" typeface="å®ä½"/>
+        <a:font script="Hant" typeface="æ°ç´°æé«"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AM94"/>
+  <dimension ref="A1:AM95"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2189,91 +2189,91 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v/>
+        <v>34</v>
       </c>
       <c r="B16" t="str">
-        <v/>
+        <v xml:space="preserve">Stacie McShane  Default - #34   </v>
       </c>
       <c r="C16" t="str">
-        <v/>
+        <v>mcshane|stacie</v>
       </c>
       <c r="D16" t="str">
-        <v/>
+        <v>NR</v>
       </c>
       <c r="E16" t="str">
-        <v/>
+        <v>0</v>
       </c>
       <c r="F16" t="str">
-        <v/>
+        <v>0.048818871</v>
       </c>
       <c r="G16" t="str">
-        <v/>
+        <v>0.057222473</v>
       </c>
       <c r="H16" t="str">
-        <v/>
+        <v>0.056958656</v>
       </c>
       <c r="I16" t="str">
-        <v/>
+        <v>0.045809234</v>
       </c>
       <c r="J16" t="str">
-        <v/>
+        <v>0.091511597</v>
       </c>
       <c r="K16" t="str">
-        <v/>
+        <v>0.052170686</v>
       </c>
       <c r="L16" t="str">
-        <v/>
+        <v>0.108439842</v>
       </c>
       <c r="M16" t="str">
-        <v/>
+        <v>0.012793303</v>
       </c>
       <c r="N16" t="str">
-        <v/>
+        <v>0.011007855</v>
       </c>
       <c r="O16" t="str">
-        <v/>
+        <v>0.015267483</v>
       </c>
       <c r="P16" t="str">
-        <v/>
+        <v>0.014969076</v>
       </c>
       <c r="Q16" t="str">
-        <v/>
+        <v>0.004118438</v>
       </c>
       <c r="R16" t="str">
-        <v/>
+        <v>0.111219491</v>
       </c>
       <c r="S16" t="str">
-        <v/>
+        <v>0.14958057</v>
       </c>
       <c r="T16" t="str">
-        <v/>
+        <v>0.002395197</v>
       </c>
       <c r="U16" t="str">
-        <v/>
+        <v>0.13223978</v>
       </c>
       <c r="V16" t="str">
-        <v/>
+        <v>0.026771651</v>
       </c>
       <c r="W16" t="str">
-        <v/>
+        <v>0.040642476</v>
       </c>
       <c r="X16" t="str">
-        <v/>
+        <v>0.018063323</v>
       </c>
       <c r="Y16" t="str">
-        <v/>
+        <v>0</v>
       </c>
       <c r="Z16" t="str">
-        <v/>
+        <v>0</v>
       </c>
       <c r="AA16" t="str">
-        <v/>
+        <v>0</v>
       </c>
       <c r="AB16" t="str">
-        <v/>
+        <v>0</v>
       </c>
       <c r="AC16" t="str">
-        <v/>
+        <v>0</v>
       </c>
       <c r="AD16" t="str">
         <v/>
@@ -2288,13 +2288,13 @@
         <v/>
       </c>
       <c r="AH16" t="str">
-        <v/>
+        <v>0.163</v>
       </c>
       <c r="AI16" t="str">
-        <v/>
+        <v>0.337</v>
       </c>
       <c r="AJ16" t="str">
-        <v/>
+        <v>0.5</v>
       </c>
       <c r="AK16" t="str">
         <v/>
@@ -2799,10 +2799,10 @@
         <v/>
       </c>
       <c r="F21" t="str">
-        <v>Salary REC</v>
+        <v/>
       </c>
       <c r="G21" t="str">
-        <v>Salary NR</v>
+        <v/>
       </c>
       <c r="H21" t="str">
         <v/>
@@ -2915,13 +2915,13 @@
         <v/>
       </c>
       <c r="E22" t="str">
-        <v>Sq Ft</v>
+        <v/>
       </c>
       <c r="F22" t="str">
-        <v>PRS</v>
+        <v>Salary REC</v>
       </c>
       <c r="G22" t="str">
-        <v>Alt PRS</v>
+        <v>Salary NR</v>
       </c>
       <c r="H22" t="str">
         <v/>
@@ -3034,13 +3034,13 @@
         <v/>
       </c>
       <c r="E23" t="str">
-        <v>8287</v>
+        <v>Sq Ft</v>
       </c>
       <c r="F23" t="str">
-        <v>0.027922382</v>
+        <v>PRS</v>
       </c>
       <c r="G23" t="str">
-        <v>0.029938151</v>
+        <v>Alt PRS</v>
       </c>
       <c r="H23" t="str">
         <v/>
@@ -3153,13 +3153,13 @@
         <v/>
       </c>
       <c r="E24" t="str">
-        <v>2280</v>
+        <v>8287</v>
       </c>
       <c r="F24" t="str">
-        <v>0.007682277</v>
+        <v>0.027922382</v>
       </c>
       <c r="G24" t="str">
-        <v>0.008236875</v>
+        <v>0.029938151</v>
       </c>
       <c r="H24" t="str">
         <v/>
@@ -3272,13 +3272,13 @@
         <v/>
       </c>
       <c r="E25" t="str">
-        <v>61572</v>
+        <v>2280</v>
       </c>
       <c r="F25" t="str">
-        <v>0.207461917</v>
+        <v>0.007682277</v>
       </c>
       <c r="G25" t="str">
-        <v>0.222438982</v>
+        <v>0.008236875</v>
       </c>
       <c r="H25" t="str">
         <v/>
@@ -3391,13 +3391,13 @@
         <v/>
       </c>
       <c r="E26" t="str">
-        <v>82809</v>
+        <v>61572</v>
       </c>
       <c r="F26" t="str">
-        <v>0.279018286</v>
+        <v>0.207461917</v>
       </c>
       <c r="G26" t="str">
-        <v>0.299161139</v>
+        <v>0.222438982</v>
       </c>
       <c r="H26" t="str">
         <v/>
@@ -3510,13 +3510,13 @@
         <v/>
       </c>
       <c r="E27" t="str">
-        <v>1326</v>
+        <v>82809</v>
       </c>
       <c r="F27" t="str">
-        <v>0.004467851</v>
+        <v>0.279018286</v>
       </c>
       <c r="G27" t="str">
-        <v>0.004790393</v>
+        <v>0.299161139</v>
       </c>
       <c r="H27" t="str">
         <v/>
@@ -3629,13 +3629,13 @@
         <v/>
       </c>
       <c r="E28" t="str">
-        <v>73209</v>
+        <v>1326</v>
       </c>
       <c r="F28" t="str">
-        <v>0.246671856</v>
+        <v>0.004467851</v>
       </c>
       <c r="G28" t="str">
-        <v>0.26447956</v>
+        <v>0.004790393</v>
       </c>
       <c r="H28" t="str">
         <v/>
@@ -3748,13 +3748,13 @@
         <v/>
       </c>
       <c r="E29" t="str">
-        <v>14821</v>
+        <v>73209</v>
       </c>
       <c r="F29" t="str">
-        <v>0.049938171</v>
+        <v>0.246671856</v>
       </c>
       <c r="G29" t="str">
-        <v>0.053543301</v>
+        <v>0.26447956</v>
       </c>
       <c r="H29" t="str">
         <v/>
@@ -3867,13 +3867,13 @@
         <v/>
       </c>
       <c r="E30" t="str">
-        <v>22500</v>
+        <v>14821</v>
       </c>
       <c r="F30" t="str">
-        <v>0.075811946</v>
+        <v>0.049938171</v>
       </c>
       <c r="G30" t="str">
-        <v>0.081284953</v>
+        <v>0.053543301</v>
       </c>
       <c r="H30" t="str">
         <v/>
@@ -3986,13 +3986,13 @@
         <v/>
       </c>
       <c r="E31" t="str">
-        <v>10000</v>
+        <v>22500</v>
       </c>
       <c r="F31" t="str">
-        <v>0.033694198</v>
+        <v>0.075811946</v>
       </c>
       <c r="G31" t="str">
-        <v>0.036126646</v>
+        <v>0.081284953</v>
       </c>
       <c r="H31" t="str">
         <v/>
@@ -4105,13 +4105,13 @@
         <v/>
       </c>
       <c r="E32" t="str">
-        <v>19983</v>
+        <v>10000</v>
       </c>
       <c r="F32" t="str">
-        <v>0.067331116</v>
+        <v>0.033694198</v>
       </c>
       <c r="G32" t="str">
-        <v>0</v>
+        <v>0.036126646</v>
       </c>
       <c r="H32" t="str">
         <v/>
@@ -4224,13 +4224,13 @@
         <v/>
       </c>
       <c r="E33" t="str">
-        <v>296787</v>
+        <v>19983</v>
       </c>
       <c r="F33" t="str">
-        <v>1</v>
+        <v>0.067331116</v>
       </c>
       <c r="G33" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H33" t="str">
         <v/>
@@ -4343,13 +4343,13 @@
         <v/>
       </c>
       <c r="E34" t="str">
-        <v/>
+        <v>296787</v>
       </c>
       <c r="F34" t="str">
-        <v/>
+        <v>1</v>
       </c>
       <c r="G34" t="str">
-        <v/>
+        <v>1</v>
       </c>
       <c r="H34" t="str">
         <v/>
@@ -4584,10 +4584,10 @@
         <v/>
       </c>
       <c r="F36" t="str">
-        <v>Salary NR</v>
+        <v/>
       </c>
       <c r="G36" t="str">
-        <v>Salary REC</v>
+        <v/>
       </c>
       <c r="H36" t="str">
         <v/>
@@ -4700,13 +4700,13 @@
         <v/>
       </c>
       <c r="E37" t="str">
-        <v>Sq Ft</v>
+        <v/>
       </c>
       <c r="F37" t="str">
-        <v>PRS</v>
+        <v>Salary NR</v>
       </c>
       <c r="G37" t="str">
-        <v>PRS</v>
+        <v>Salary REC</v>
       </c>
       <c r="H37" t="str">
         <v/>
@@ -4819,13 +4819,13 @@
         <v/>
       </c>
       <c r="E38" t="str">
-        <v>54008</v>
+        <v>Sq Ft</v>
       </c>
       <c r="F38" t="str">
-        <v>0.135932447</v>
+        <v>PRS</v>
       </c>
       <c r="G38" t="str">
-        <v>0.14238298</v>
+        <v>PRS</v>
       </c>
       <c r="H38" t="str">
         <v/>
@@ -4938,13 +4938,13 @@
         <v/>
       </c>
       <c r="E39" t="str">
-        <v>107890</v>
+        <v>54008</v>
       </c>
       <c r="F39" t="str">
-        <v>0.271547764</v>
+        <v>0.135932447</v>
       </c>
       <c r="G39" t="str">
-        <v>0.284433782</v>
+        <v>0.14238298</v>
       </c>
       <c r="H39" t="str">
         <v/>
@@ -5057,13 +5057,13 @@
         <v/>
       </c>
       <c r="E40" t="str">
-        <v>61508</v>
+        <v>107890</v>
       </c>
       <c r="F40" t="str">
-        <v>0.154809156</v>
+        <v>0.271547764</v>
       </c>
       <c r="G40" t="str">
-        <v>0.162155464</v>
+        <v>0.284433782</v>
       </c>
       <c r="H40" t="str">
         <v/>
@@ -5176,13 +5176,13 @@
         <v/>
       </c>
       <c r="E41" t="str">
-        <v>127848</v>
+        <v>61508</v>
       </c>
       <c r="F41" t="str">
-        <v>0.321779948</v>
+        <v>0.154809156</v>
       </c>
       <c r="G41" t="str">
-        <v>0.337049682</v>
+        <v>0.162155464</v>
       </c>
       <c r="H41" t="str">
         <v/>
@@ -5295,13 +5295,13 @@
         <v/>
       </c>
       <c r="E42" t="str">
-        <v>15083</v>
+        <v>127848</v>
       </c>
       <c r="F42" t="str">
-        <v>0.037962322</v>
+        <v>0.321779948</v>
       </c>
       <c r="G42" t="str">
-        <v>0.039763785</v>
+        <v>0.337049682</v>
       </c>
       <c r="H42" t="str">
         <v/>
@@ -5414,13 +5414,13 @@
         <v/>
       </c>
       <c r="E43" t="str">
-        <v>12978</v>
+        <v>15083</v>
       </c>
       <c r="F43" t="str">
-        <v>0.032664259</v>
+        <v>0.037962322</v>
       </c>
       <c r="G43" t="str">
-        <v>0.034214307</v>
+        <v>0.039763785</v>
       </c>
       <c r="H43" t="str">
         <v/>
@@ -5533,13 +5533,13 @@
         <v/>
       </c>
       <c r="E44" t="str">
-        <v>18000</v>
+        <v>12978</v>
       </c>
       <c r="F44" t="str">
-        <v>0.045304104</v>
+        <v>0.032664259</v>
       </c>
       <c r="G44" t="str">
-        <v>0</v>
+        <v>0.034214307</v>
       </c>
       <c r="H44" t="str">
         <v/>
@@ -5652,13 +5652,13 @@
         <v/>
       </c>
       <c r="E45" t="str">
-        <v>397315</v>
+        <v>18000</v>
       </c>
       <c r="F45" t="str">
-        <v>1</v>
+        <v>0.045304104</v>
       </c>
       <c r="G45" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H45" t="str">
         <v/>
@@ -5771,13 +5771,13 @@
         <v/>
       </c>
       <c r="E46" t="str">
-        <v/>
+        <v>397315</v>
       </c>
       <c r="F46" t="str">
-        <v/>
+        <v>1</v>
       </c>
       <c r="G46" t="str">
-        <v/>
+        <v>1</v>
       </c>
       <c r="H46" t="str">
         <v/>
@@ -6009,10 +6009,10 @@
         <v/>
       </c>
       <c r="E48" t="str">
-        <v>Sq Ft</v>
+        <v/>
       </c>
       <c r="F48" t="str">
-        <v>PRS</v>
+        <v/>
       </c>
       <c r="G48" t="str">
         <v/>
@@ -6128,10 +6128,10 @@
         <v/>
       </c>
       <c r="E49" t="str">
-        <v>41821</v>
+        <v>Sq Ft</v>
       </c>
       <c r="F49" t="str">
-        <v>0.299502274</v>
+        <v>PRS</v>
       </c>
       <c r="G49" t="str">
         <v/>
@@ -6247,10 +6247,10 @@
         <v/>
       </c>
       <c r="E50" t="str">
-        <v>49020</v>
+        <v>41821</v>
       </c>
       <c r="F50" t="str">
-        <v>0.351058116</v>
+        <v>0.299502274</v>
       </c>
       <c r="G50" t="str">
         <v/>
@@ -6366,10 +6366,10 @@
         <v/>
       </c>
       <c r="E51" t="str">
-        <v>48794</v>
+        <v>49020</v>
       </c>
       <c r="F51" t="str">
-        <v>0.34943961</v>
+        <v>0.351058116</v>
       </c>
       <c r="G51" t="str">
         <v/>
@@ -6485,10 +6485,10 @@
         <v/>
       </c>
       <c r="E52" t="str">
-        <v>139635</v>
+        <v>48794</v>
       </c>
       <c r="F52" t="str">
-        <v>1</v>
+        <v>0.34943961</v>
       </c>
       <c r="G52" t="str">
         <v/>
@@ -6604,10 +6604,10 @@
         <v/>
       </c>
       <c r="E53" t="str">
-        <v/>
+        <v>139635</v>
       </c>
       <c r="F53" t="str">
-        <v/>
+        <v>1</v>
       </c>
       <c r="G53" t="str">
         <v/>
@@ -6842,7 +6842,7 @@
         <v/>
       </c>
       <c r="E55" t="str">
-        <v>0.463</v>
+        <v/>
       </c>
       <c r="F55" t="str">
         <v/>
@@ -6961,7 +6961,7 @@
         <v/>
       </c>
       <c r="E56" t="str">
-        <v>0.337</v>
+        <v>0.463</v>
       </c>
       <c r="F56" t="str">
         <v/>
@@ -7080,7 +7080,7 @@
         <v/>
       </c>
       <c r="E57" t="str">
-        <v>0.2</v>
+        <v>0.337</v>
       </c>
       <c r="F57" t="str">
         <v/>
@@ -7199,7 +7199,7 @@
         <v/>
       </c>
       <c r="E58" t="str">
-        <v/>
+        <v>0.2</v>
       </c>
       <c r="F58" t="str">
         <v/>
@@ -8029,10 +8029,10 @@
         <v/>
       </c>
       <c r="D65" t="str">
-        <v>8568.95</v>
+        <v/>
       </c>
       <c r="E65" t="str">
-        <v>Insert $</v>
+        <v/>
       </c>
       <c r="F65" t="str">
         <v/>
@@ -8148,10 +8148,10 @@
         <v/>
       </c>
       <c r="D66" t="str">
-        <v xml:space="preserve">Gregory Masciantonio  Default - #19   </v>
+        <v>8568.95</v>
       </c>
       <c r="E66" t="str">
-        <v>Employee</v>
+        <v>Insert $</v>
       </c>
       <c r="F66" t="str">
         <v/>
@@ -8267,10 +8267,10 @@
         <v/>
       </c>
       <c r="D67" t="str">
-        <v/>
+        <v xml:space="preserve">Gregory Masciantonio  Default - #19   </v>
       </c>
       <c r="E67" t="str">
-        <v/>
+        <v>Employee</v>
       </c>
       <c r="F67" t="str">
         <v/>
@@ -8380,16 +8380,16 @@
         <v/>
       </c>
       <c r="B68" t="str">
-        <v xml:space="preserve"> Property Code</v>
+        <v/>
       </c>
       <c r="C68" t="str">
-        <v>Property Name</v>
+        <v/>
       </c>
       <c r="D68" t="str">
-        <v>% Alloc</v>
+        <v/>
       </c>
       <c r="E68" t="str">
-        <v>$ Alloc</v>
+        <v/>
       </c>
       <c r="F68" t="str">
         <v/>
@@ -8499,16 +8499,16 @@
         <v/>
       </c>
       <c r="B69" t="str">
-        <v>2010</v>
+        <v xml:space="preserve"> Property Code</v>
       </c>
       <c r="C69" t="str">
-        <v>LIK</v>
+        <v>Property Name</v>
       </c>
       <c r="D69" t="str">
-        <v>0</v>
+        <v>% Alloc</v>
       </c>
       <c r="E69" t="str">
-        <v>0</v>
+        <v>$ Alloc</v>
       </c>
       <c r="F69" t="str">
         <v/>
@@ -8618,16 +8618,16 @@
         <v/>
       </c>
       <c r="B70" t="str">
-        <v>3610</v>
+        <v>2010</v>
       </c>
       <c r="C70" t="str">
-        <v>Building 1</v>
+        <v>LIK</v>
       </c>
       <c r="D70" t="str">
-        <v>0.063464532</v>
+        <v>0</v>
       </c>
       <c r="E70" t="str">
-        <v>543.8243999</v>
+        <v>0</v>
       </c>
       <c r="F70" t="str">
         <v/>
@@ -8737,16 +8737,16 @@
         <v/>
       </c>
       <c r="B71" t="str">
-        <v>3620</v>
+        <v>3610</v>
       </c>
       <c r="C71" t="str">
-        <v>Building 2</v>
+        <v>Building 1</v>
       </c>
       <c r="D71" t="str">
-        <v>0.074389215</v>
+        <v>0.063464532</v>
       </c>
       <c r="E71" t="str">
-        <v>637.4374616</v>
+        <v>543.8243999</v>
       </c>
       <c r="F71" t="str">
         <v/>
@@ -8856,16 +8856,16 @@
         <v/>
       </c>
       <c r="B72" t="str">
-        <v>3640</v>
+        <v>3620</v>
       </c>
       <c r="C72" t="str">
-        <v>Building 4</v>
+        <v>Building 2</v>
       </c>
       <c r="D72" t="str">
-        <v>0.074046253</v>
+        <v>0.074389215</v>
       </c>
       <c r="E72" t="str">
-        <v>634.4986435</v>
+        <v>637.4374616</v>
       </c>
       <c r="F72" t="str">
         <v/>
@@ -8975,16 +8975,16 @@
         <v/>
       </c>
       <c r="B73" t="str">
-        <v>4050</v>
+        <v>3640</v>
       </c>
       <c r="C73" t="str">
-        <v>Building 5</v>
+        <v>Building 4</v>
       </c>
       <c r="D73" t="str">
-        <v>0.062377983</v>
+        <v>0.074046253</v>
       </c>
       <c r="E73" t="str">
-        <v>534.5138215</v>
+        <v>634.4986435</v>
       </c>
       <c r="F73" t="str">
         <v/>
@@ -9094,16 +9094,16 @@
         <v/>
       </c>
       <c r="B74" t="str">
-        <v>4060</v>
+        <v>4050</v>
       </c>
       <c r="C74" t="str">
-        <v>Building 6</v>
+        <v>Building 5</v>
       </c>
       <c r="D74" t="str">
-        <v>0.12461044</v>
+        <v>0.062377983</v>
       </c>
       <c r="E74" t="str">
-        <v>1067.780629</v>
+        <v>534.5138215</v>
       </c>
       <c r="F74" t="str">
         <v/>
@@ -9213,16 +9213,16 @@
         <v/>
       </c>
       <c r="B75" t="str">
-        <v>4070</v>
+        <v>4060</v>
       </c>
       <c r="C75" t="str">
-        <v>Building 7</v>
+        <v>Building 6</v>
       </c>
       <c r="D75" t="str">
-        <v>0.071040309</v>
+        <v>0.12461044</v>
       </c>
       <c r="E75" t="str">
-        <v>608.7408556</v>
+        <v>1067.780629</v>
       </c>
       <c r="F75" t="str">
         <v/>
@@ -9332,16 +9332,16 @@
         <v/>
       </c>
       <c r="B76" t="str">
-        <v>4080</v>
+        <v>4070</v>
       </c>
       <c r="C76" t="str">
-        <v>Building 8</v>
+        <v>Building 7</v>
       </c>
       <c r="D76" t="str">
-        <v>0.147661466</v>
+        <v>0.071040309</v>
       </c>
       <c r="E76" t="str">
-        <v>1265.303715</v>
+        <v>608.7408556</v>
       </c>
       <c r="F76" t="str">
         <v/>
@@ -9451,16 +9451,16 @@
         <v/>
       </c>
       <c r="B77" t="str">
-        <v>40A0</v>
+        <v>4080</v>
       </c>
       <c r="C77" t="str">
-        <v>Building A</v>
+        <v>Building 8</v>
       </c>
       <c r="D77" t="str">
-        <v>0.017420514</v>
+        <v>0.147661466</v>
       </c>
       <c r="E77" t="str">
-        <v>149.2755142</v>
+        <v>1265.303715</v>
       </c>
       <c r="F77" t="str">
         <v/>
@@ -9570,16 +9570,16 @@
         <v/>
       </c>
       <c r="B78" t="str">
-        <v>40B0</v>
+        <v>40A0</v>
       </c>
       <c r="C78" t="str">
-        <v>Building B</v>
+        <v>Building A</v>
       </c>
       <c r="D78" t="str">
-        <v>0.014989288</v>
+        <v>0.017420514</v>
       </c>
       <c r="E78" t="str">
-        <v>128.4424599</v>
+        <v>149.2755142</v>
       </c>
       <c r="F78" t="str">
         <v/>
@@ -9689,16 +9689,16 @@
         <v/>
       </c>
       <c r="B79" t="str">
-        <v>40C0</v>
+        <v>40B0</v>
       </c>
       <c r="C79" t="str">
-        <v>Building C</v>
+        <v>Building B</v>
       </c>
       <c r="D79" t="str">
-        <v>0</v>
+        <v>0.014989288</v>
       </c>
       <c r="E79" t="str">
-        <v>0</v>
+        <v>128.4424599</v>
       </c>
       <c r="F79" t="str">
         <v/>
@@ -9808,16 +9808,16 @@
         <v/>
       </c>
       <c r="B80" t="str">
-        <v>1100</v>
+        <v>40C0</v>
       </c>
       <c r="C80" t="str">
-        <v>Parkwood Professional</v>
+        <v>Building C</v>
       </c>
       <c r="D80" t="str">
-        <v>0.009772834</v>
+        <v>0</v>
       </c>
       <c r="E80" t="str">
-        <v>83.74292347</v>
+        <v>0</v>
       </c>
       <c r="F80" t="str">
         <v/>
@@ -9927,16 +9927,16 @@
         <v/>
       </c>
       <c r="B81" t="str">
-        <v>1500</v>
+        <v>1100</v>
       </c>
       <c r="C81" t="str">
-        <v>Eastwick</v>
+        <v>Parkwood Professional</v>
       </c>
       <c r="D81" t="str">
-        <v>0.002688797</v>
+        <v>0.009772834</v>
       </c>
       <c r="E81" t="str">
-        <v>23.04016719</v>
+        <v>83.74292347</v>
       </c>
       <c r="F81" t="str">
         <v/>
@@ -10046,16 +10046,16 @@
         <v/>
       </c>
       <c r="B82" t="str">
-        <v>2300</v>
+        <v>1500</v>
       </c>
       <c r="C82" t="str">
-        <v>Brookwood SC</v>
+        <v>Eastwick</v>
       </c>
       <c r="D82" t="str">
-        <v>0.072611671</v>
+        <v>0.002688797</v>
       </c>
       <c r="E82" t="str">
-        <v>622.2057782</v>
+        <v>23.04016719</v>
       </c>
       <c r="F82" t="str">
         <v/>
@@ -10165,16 +10165,16 @@
         <v/>
       </c>
       <c r="B83" t="str">
-        <v>4500</v>
+        <v>2300</v>
       </c>
       <c r="C83" t="str">
-        <v>Grays Ferry SC</v>
+        <v>Brookwood SC</v>
       </c>
       <c r="D83" t="str">
-        <v>0.0976564</v>
+        <v>0.072611671</v>
       </c>
       <c r="E83" t="str">
-        <v>836.8128092</v>
+        <v>622.2057782</v>
       </c>
       <c r="F83" t="str">
         <v/>
@@ -10284,16 +10284,16 @@
         <v/>
       </c>
       <c r="B84" t="str">
-        <v>5600</v>
+        <v>4500</v>
       </c>
       <c r="C84" t="str">
-        <v>HK Co Castor Ave</v>
+        <v>Grays Ferry SC</v>
       </c>
       <c r="D84" t="str">
-        <v>0.001563748</v>
+        <v>0.0976564</v>
       </c>
       <c r="E84" t="str">
-        <v>13.39967618</v>
+        <v>836.8128092</v>
       </c>
       <c r="F84" t="str">
         <v/>
@@ -10403,16 +10403,16 @@
         <v/>
       </c>
       <c r="B85" t="str">
-        <v>7010</v>
+        <v>5600</v>
       </c>
       <c r="C85" t="str">
-        <v>Parkwood SC</v>
+        <v>HK Co Castor Ave</v>
       </c>
       <c r="D85" t="str">
-        <v>0.086335149</v>
+        <v>0.001563748</v>
       </c>
       <c r="E85" t="str">
-        <v>739.8015789</v>
+        <v>13.39967618</v>
       </c>
       <c r="F85" t="str">
         <v/>
@@ -10522,16 +10522,16 @@
         <v/>
       </c>
       <c r="B86" t="str">
-        <v>7200</v>
+        <v>7010</v>
       </c>
       <c r="C86" t="str">
-        <v>Elbridge SC</v>
+        <v>Parkwood SC</v>
       </c>
       <c r="D86" t="str">
-        <v>0.01747836</v>
+        <v>0.086335149</v>
       </c>
       <c r="E86" t="str">
-        <v>149.7711921</v>
+        <v>739.8015789</v>
       </c>
       <c r="F86" t="str">
         <v/>
@@ -10641,16 +10641,16 @@
         <v/>
       </c>
       <c r="B87" t="str">
-        <v>7300</v>
+        <v>7200</v>
       </c>
       <c r="C87" t="str">
-        <v>Revere SC</v>
+        <v>Elbridge SC</v>
       </c>
       <c r="D87" t="str">
-        <v>0.026534181</v>
+        <v>0.01747836</v>
       </c>
       <c r="E87" t="str">
-        <v>227.370071</v>
+        <v>149.7711921</v>
       </c>
       <c r="F87" t="str">
         <v/>
@@ -10760,16 +10760,16 @@
         <v/>
       </c>
       <c r="B88" t="str">
-        <v>8200</v>
+        <v>7300</v>
       </c>
       <c r="C88" t="str">
-        <v>Trust #4</v>
+        <v>Revere SC</v>
       </c>
       <c r="D88" t="str">
-        <v>0.011792969</v>
+        <v>0.026534181</v>
       </c>
       <c r="E88" t="str">
-        <v>101.0533649</v>
+        <v>227.370071</v>
       </c>
       <c r="F88" t="str">
         <v/>
@@ -10879,16 +10879,16 @@
         <v/>
       </c>
       <c r="B89" t="str">
-        <v>9510</v>
+        <v>8200</v>
       </c>
       <c r="C89" t="str">
-        <v>Lafayette Hill SC</v>
+        <v>Trust #4</v>
       </c>
       <c r="D89" t="str">
-        <v>0.023565891</v>
+        <v>0.011792969</v>
       </c>
       <c r="E89" t="str">
-        <v>201.934939</v>
+        <v>101.0533649</v>
       </c>
       <c r="F89" t="str">
         <v/>
@@ -10998,16 +10998,16 @@
         <v/>
       </c>
       <c r="B90" t="str">
-        <v>4900</v>
+        <v>9510</v>
       </c>
       <c r="C90" t="str">
-        <v>Office Works</v>
+        <v>Lafayette Hill SC</v>
       </c>
       <c r="D90" t="str">
-        <v>0</v>
+        <v>0.023565891</v>
       </c>
       <c r="E90" t="str">
-        <v>0</v>
+        <v>201.934939</v>
       </c>
       <c r="F90" t="str">
         <v/>
@@ -11117,10 +11117,10 @@
         <v/>
       </c>
       <c r="B91" t="str">
-        <v>Marketing</v>
+        <v>4900</v>
       </c>
       <c r="C91" t="str">
-        <v>Marketing</v>
+        <v>Office Works</v>
       </c>
       <c r="D91" t="str">
         <v>0</v>
@@ -11236,10 +11236,10 @@
         <v/>
       </c>
       <c r="B92" t="str">
-        <v>0800</v>
+        <v>Marketing</v>
       </c>
       <c r="C92" t="str">
-        <v>Bellmawr</v>
+        <v>Marketing</v>
       </c>
       <c r="D92" t="str">
         <v>0</v>
@@ -11355,10 +11355,10 @@
         <v/>
       </c>
       <c r="B93" t="str">
-        <v>Eastwick</v>
+        <v>0800</v>
       </c>
       <c r="C93" t="str">
-        <v>Eastwick JV</v>
+        <v>Bellmawr</v>
       </c>
       <c r="D93" t="str">
         <v>0</v>
@@ -11474,123 +11474,242 @@
         <v/>
       </c>
       <c r="B94" t="str">
-        <v/>
+        <v>Eastwick</v>
       </c>
       <c r="C94" t="str">
-        <v/>
+        <v>Eastwick JV</v>
       </c>
       <c r="D94" t="str">
+        <v>0</v>
+      </c>
+      <c r="E94" t="str">
+        <v>0</v>
+      </c>
+      <c r="F94" t="str">
+        <v/>
+      </c>
+      <c r="G94" t="str">
+        <v/>
+      </c>
+      <c r="H94" t="str">
+        <v/>
+      </c>
+      <c r="I94" t="str">
+        <v/>
+      </c>
+      <c r="J94" t="str">
+        <v/>
+      </c>
+      <c r="K94" t="str">
+        <v/>
+      </c>
+      <c r="L94" t="str">
+        <v/>
+      </c>
+      <c r="M94" t="str">
+        <v/>
+      </c>
+      <c r="N94" t="str">
+        <v/>
+      </c>
+      <c r="O94" t="str">
+        <v/>
+      </c>
+      <c r="P94" t="str">
+        <v/>
+      </c>
+      <c r="Q94" t="str">
+        <v/>
+      </c>
+      <c r="R94" t="str">
+        <v/>
+      </c>
+      <c r="S94" t="str">
+        <v/>
+      </c>
+      <c r="T94" t="str">
+        <v/>
+      </c>
+      <c r="U94" t="str">
+        <v/>
+      </c>
+      <c r="V94" t="str">
+        <v/>
+      </c>
+      <c r="W94" t="str">
+        <v/>
+      </c>
+      <c r="X94" t="str">
+        <v/>
+      </c>
+      <c r="Y94" t="str">
+        <v/>
+      </c>
+      <c r="Z94" t="str">
+        <v/>
+      </c>
+      <c r="AA94" t="str">
+        <v/>
+      </c>
+      <c r="AB94" t="str">
+        <v/>
+      </c>
+      <c r="AC94" t="str">
+        <v/>
+      </c>
+      <c r="AD94" t="str">
+        <v/>
+      </c>
+      <c r="AE94" t="str">
+        <v/>
+      </c>
+      <c r="AF94" t="str">
+        <v/>
+      </c>
+      <c r="AG94" t="str">
+        <v/>
+      </c>
+      <c r="AH94" t="str">
+        <v/>
+      </c>
+      <c r="AI94" t="str">
+        <v/>
+      </c>
+      <c r="AJ94" t="str">
+        <v/>
+      </c>
+      <c r="AK94" t="str">
+        <v/>
+      </c>
+      <c r="AL94" t="str">
+        <v/>
+      </c>
+      <c r="AM94" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="str">
+        <v/>
+      </c>
+      <c r="B95" t="str">
+        <v/>
+      </c>
+      <c r="C95" t="str">
+        <v/>
+      </c>
+      <c r="D95" t="str">
         <v>1</v>
       </c>
-      <c r="E94" t="str">
+      <c r="E95" t="str">
         <v>8568.95</v>
       </c>
-      <c r="F94" t="str">
-        <v/>
-      </c>
-      <c r="G94" t="str">
-        <v/>
-      </c>
-      <c r="H94" t="str">
-        <v/>
-      </c>
-      <c r="I94" t="str">
-        <v/>
-      </c>
-      <c r="J94" t="str">
-        <v/>
-      </c>
-      <c r="K94" t="str">
-        <v/>
-      </c>
-      <c r="L94" t="str">
-        <v/>
-      </c>
-      <c r="M94" t="str">
-        <v/>
-      </c>
-      <c r="N94" t="str">
-        <v/>
-      </c>
-      <c r="O94" t="str">
-        <v/>
-      </c>
-      <c r="P94" t="str">
-        <v/>
-      </c>
-      <c r="Q94" t="str">
-        <v/>
-      </c>
-      <c r="R94" t="str">
-        <v/>
-      </c>
-      <c r="S94" t="str">
-        <v/>
-      </c>
-      <c r="T94" t="str">
-        <v/>
-      </c>
-      <c r="U94" t="str">
-        <v/>
-      </c>
-      <c r="V94" t="str">
-        <v/>
-      </c>
-      <c r="W94" t="str">
-        <v/>
-      </c>
-      <c r="X94" t="str">
-        <v/>
-      </c>
-      <c r="Y94" t="str">
-        <v/>
-      </c>
-      <c r="Z94" t="str">
-        <v/>
-      </c>
-      <c r="AA94" t="str">
-        <v/>
-      </c>
-      <c r="AB94" t="str">
-        <v/>
-      </c>
-      <c r="AC94" t="str">
-        <v/>
-      </c>
-      <c r="AD94" t="str">
-        <v/>
-      </c>
-      <c r="AE94" t="str">
-        <v/>
-      </c>
-      <c r="AF94" t="str">
-        <v/>
-      </c>
-      <c r="AG94" t="str">
-        <v/>
-      </c>
-      <c r="AH94" t="str">
-        <v/>
-      </c>
-      <c r="AI94" t="str">
-        <v/>
-      </c>
-      <c r="AJ94" t="str">
-        <v/>
-      </c>
-      <c r="AK94" t="str">
-        <v/>
-      </c>
-      <c r="AL94" t="str">
-        <v/>
-      </c>
-      <c r="AM94" t="str">
+      <c r="F95" t="str">
+        <v/>
+      </c>
+      <c r="G95" t="str">
+        <v/>
+      </c>
+      <c r="H95" t="str">
+        <v/>
+      </c>
+      <c r="I95" t="str">
+        <v/>
+      </c>
+      <c r="J95" t="str">
+        <v/>
+      </c>
+      <c r="K95" t="str">
+        <v/>
+      </c>
+      <c r="L95" t="str">
+        <v/>
+      </c>
+      <c r="M95" t="str">
+        <v/>
+      </c>
+      <c r="N95" t="str">
+        <v/>
+      </c>
+      <c r="O95" t="str">
+        <v/>
+      </c>
+      <c r="P95" t="str">
+        <v/>
+      </c>
+      <c r="Q95" t="str">
+        <v/>
+      </c>
+      <c r="R95" t="str">
+        <v/>
+      </c>
+      <c r="S95" t="str">
+        <v/>
+      </c>
+      <c r="T95" t="str">
+        <v/>
+      </c>
+      <c r="U95" t="str">
+        <v/>
+      </c>
+      <c r="V95" t="str">
+        <v/>
+      </c>
+      <c r="W95" t="str">
+        <v/>
+      </c>
+      <c r="X95" t="str">
+        <v/>
+      </c>
+      <c r="Y95" t="str">
+        <v/>
+      </c>
+      <c r="Z95" t="str">
+        <v/>
+      </c>
+      <c r="AA95" t="str">
+        <v/>
+      </c>
+      <c r="AB95" t="str">
+        <v/>
+      </c>
+      <c r="AC95" t="str">
+        <v/>
+      </c>
+      <c r="AD95" t="str">
+        <v/>
+      </c>
+      <c r="AE95" t="str">
+        <v/>
+      </c>
+      <c r="AF95" t="str">
+        <v/>
+      </c>
+      <c r="AG95" t="str">
+        <v/>
+      </c>
+      <c r="AH95" t="str">
+        <v/>
+      </c>
+      <c r="AI95" t="str">
+        <v/>
+      </c>
+      <c r="AJ95" t="str">
+        <v/>
+      </c>
+      <c r="AK95" t="str">
+        <v/>
+      </c>
+      <c r="AL95" t="str">
+        <v/>
+      </c>
+      <c r="AM95" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AM94"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AM95"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>